<commit_message>
Added 100 new coins
</commit_message>
<xml_diff>
--- a/Opponent_Tracker.xlsx
+++ b/Opponent_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{946EBDB1-D282-4615-9CA1-B6EEA768A8C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA05E1AD-3B53-4FAE-BDA4-A167EEA6F441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7155" yWindow="1710" windowWidth="14400" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="opponents_table" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="152">
   <si>
     <t>Opponent</t>
   </si>
@@ -464,6 +464,18 @@
   </si>
   <si>
     <t>Solid Workers</t>
+  </si>
+  <si>
+    <t>Shady Character Owen</t>
+  </si>
+  <si>
+    <t>Thunder Rush</t>
+  </si>
+  <si>
+    <t>Shady Character Bernard</t>
+  </si>
+  <si>
+    <t>Neverending Flames</t>
   </si>
 </sst>
 </file>
@@ -675,6 +687,12 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -691,14 +709,8 @@
     <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1042,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -1051,26 +1063,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25" t="s">
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25" t="s">
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25" t="s">
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
     </row>
     <row r="2" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
@@ -1237,40 +1249,40 @@
       <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="28">
         <v>8</v>
       </c>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="29">
-        <v>15</v>
-      </c>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="27">
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="31">
+        <v>15</v>
+      </c>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="29">
         <v>19</v>
       </c>
-      <c r="J6" s="28"/>
-      <c r="K6" s="28"/>
-      <c r="L6" s="32"/>
-      <c r="M6" s="32"/>
-      <c r="N6" s="32"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="33"/>
     </row>
     <row r="7" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="30">
+      <c r="C7" s="32">
         <v>42</v>
       </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="28"/>
-      <c r="K7" s="28"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
     </row>
     <row r="8" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1981,7 +1993,7 @@
       <c r="L58" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="M58" s="31" t="s">
+      <c r="M58" s="25" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2006,7 +2018,7 @@
       <c r="L60" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="M60" s="31" t="s">
+      <c r="M60" s="25" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2031,7 +2043,7 @@
       <c r="L62" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="M62" s="31" t="s">
+      <c r="M62" s="25" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2045,7 +2057,7 @@
       <c r="L63" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="M63" s="31" t="s">
+      <c r="M63" s="25" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2067,10 +2079,10 @@
       <c r="B65" t="s">
         <v>135</v>
       </c>
-      <c r="M65" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="N65" s="33" t="s">
+      <c r="M65" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N65" s="26" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2081,7 +2093,7 @@
       <c r="B66" t="s">
         <v>137</v>
       </c>
-      <c r="M66" s="31" t="s">
+      <c r="M66" s="25" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2092,7 +2104,7 @@
       <c r="B67" t="s">
         <v>139</v>
       </c>
-      <c r="M67" s="31" t="s">
+      <c r="M67" s="25" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2103,10 +2115,10 @@
       <c r="B68" t="s">
         <v>141</v>
       </c>
-      <c r="M68" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="N68" s="33" t="s">
+      <c r="M68" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N68" s="26" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2117,10 +2129,10 @@
       <c r="B69" t="s">
         <v>143</v>
       </c>
-      <c r="M69" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="N69" s="33" t="s">
+      <c r="M69" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N69" s="26" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2131,7 +2143,7 @@
       <c r="B70" t="s">
         <v>145</v>
       </c>
-      <c r="M70" s="31" t="s">
+      <c r="M70" s="25" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2142,10 +2154,32 @@
       <c r="B71" t="s">
         <v>147</v>
       </c>
-      <c r="M71" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="N71" s="33" t="s">
+      <c r="M71" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N71" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>148</v>
+      </c>
+      <c r="B72" t="s">
+        <v>149</v>
+      </c>
+      <c r="N72" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>150</v>
+      </c>
+      <c r="B73" t="s">
+        <v>151</v>
+      </c>
+      <c r="N73" s="26" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added majority of opponents to Verdant forest day eve night 4 and day eve 5
</commit_message>
<xml_diff>
--- a/Opponent_Tracker.xlsx
+++ b/Opponent_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA05E1AD-3B53-4FAE-BDA4-A167EEA6F441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B45039-599A-485E-B279-47A4CCF1E17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7155" yWindow="1710" windowWidth="14400" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="opponents_table" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="191">
   <si>
     <t>Opponent</t>
   </si>
@@ -476,6 +476,123 @@
   </si>
   <si>
     <t>Neverending Flames</t>
+  </si>
+  <si>
+    <t>Ghost Whisperer Vera</t>
+  </si>
+  <si>
+    <t>Terrible Nightmares</t>
+  </si>
+  <si>
+    <t>Police Constable Floyd</t>
+  </si>
+  <si>
+    <t>Police Sergeant Douglas</t>
+  </si>
+  <si>
+    <t>Peace Keepers</t>
+  </si>
+  <si>
+    <t>Energy Beams</t>
+  </si>
+  <si>
+    <t>Scavenge And Retreat</t>
+  </si>
+  <si>
+    <t>Rocket Grunt Margot</t>
+  </si>
+  <si>
+    <t>Day 5</t>
+  </si>
+  <si>
+    <t>Eve 5</t>
+  </si>
+  <si>
+    <t>Night 5</t>
+  </si>
+  <si>
+    <t>Psychic Nova</t>
+  </si>
+  <si>
+    <t>Telekinesis</t>
+  </si>
+  <si>
+    <t>Nature Lover Erin</t>
+  </si>
+  <si>
+    <t>Young Sage Kai</t>
+  </si>
+  <si>
+    <t>Forest Guardians</t>
+  </si>
+  <si>
+    <t>Thunder Ball</t>
+  </si>
+  <si>
+    <t>Youngster Cooper</t>
+  </si>
+  <si>
+    <t>Solid Dynamite</t>
+  </si>
+  <si>
+    <t>Gambler Victor</t>
+  </si>
+  <si>
+    <t>Risky Flips</t>
+  </si>
+  <si>
+    <t>Old Traveller Harold</t>
+  </si>
+  <si>
+    <t>Old Traveller Cliff</t>
+  </si>
+  <si>
+    <t>Hard Hitters</t>
+  </si>
+  <si>
+    <t>Solid Invertebrates</t>
+  </si>
+  <si>
+    <t>Clown Hubert</t>
+  </si>
+  <si>
+    <t>Scary Phobias</t>
+  </si>
+  <si>
+    <t>Clown Glenn</t>
+  </si>
+  <si>
+    <t>Strange Damage Counters</t>
+  </si>
+  <si>
+    <t>Rocket Exec Proton</t>
+  </si>
+  <si>
+    <t>Rocket Exec Petrel</t>
+  </si>
+  <si>
+    <t>Rocket Exec Ariana</t>
+  </si>
+  <si>
+    <t>Rocket Exec Archer</t>
+  </si>
+  <si>
+    <t>Under The Shadow Of Wings</t>
+  </si>
+  <si>
+    <t>Relentless Poison</t>
+  </si>
+  <si>
+    <t>Forced Evolutions</t>
+  </si>
+  <si>
+    <t>Jet Shell</t>
+  </si>
+  <si>
+    <t>Rocket Boss Giovanni</t>
+  </si>
+  <si>
+    <t>Rocket Psychic Supremacy</t>
   </si>
 </sst>
 </file>
@@ -499,7 +616,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -602,6 +719,36 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF55FE00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3FBFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC901"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC600EE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC3EA00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -615,7 +762,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -693,8 +840,26 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -706,11 +871,11 @@
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -720,6 +885,12 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFC901"/>
+      <color rgb="FF3FBFFF"/>
+      <color rgb="FFC3EA00"/>
+      <color rgb="FFC600EE"/>
+      <color rgb="FFFFED01"/>
+      <color rgb="FF55FE00"/>
       <color rgb="FF6600CC"/>
       <color rgb="FFFF6600"/>
       <color rgb="FF2D55FF"/>
@@ -1054,7 +1225,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:Q91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -1062,29 +1233,34 @@
     <col min="3" max="8" width="7.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C1" s="27" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C1" s="32" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27" t="s">
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27" t="s">
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32" t="s">
         <v>130</v>
       </c>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27" t="s">
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32" t="s">
         <v>131</v>
       </c>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-    </row>
-    <row r="2" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="32" t="s">
+        <v>131</v>
+      </c>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="32"/>
+    </row>
+    <row r="2" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -1127,8 +1303,17 @@
       <c r="N2" s="23" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O2" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="P2" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q2" s="29" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1160,14 +1345,25 @@
         <v>4</v>
       </c>
       <c r="L3" s="21">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M3" s="22">
         <v>7</v>
       </c>
-      <c r="N3" s="23"/>
-    </row>
-    <row r="4" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N3" s="23">
+        <v>5</v>
+      </c>
+      <c r="O3" s="27">
+        <v>7</v>
+      </c>
+      <c r="P3" s="28">
+        <v>7</v>
+      </c>
+      <c r="Q3" s="29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1204,9 +1400,20 @@
       <c r="M4" s="22">
         <v>7</v>
       </c>
-      <c r="N4" s="23"/>
-    </row>
-    <row r="5" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N4" s="23">
+        <v>0</v>
+      </c>
+      <c r="O4" s="27">
+        <v>7</v>
+      </c>
+      <c r="P4" s="28">
+        <v>7</v>
+      </c>
+      <c r="Q4" s="29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1238,54 +1445,78 @@
         <v>15</v>
       </c>
       <c r="L5" s="21">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M5" s="22">
         <v>11</v>
       </c>
-      <c r="N5" s="23"/>
-    </row>
-    <row r="6" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N5" s="23">
+        <v>9</v>
+      </c>
+      <c r="O5" s="27">
+        <v>19</v>
+      </c>
+      <c r="P5" s="28">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="28">
+      <c r="C6" s="34">
         <v>8</v>
       </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="31">
-        <v>15</v>
-      </c>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="29">
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="37">
+        <v>15</v>
+      </c>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="35">
         <v>19</v>
       </c>
-      <c r="J6" s="30"/>
-      <c r="K6" s="30"/>
-      <c r="L6" s="33"/>
-      <c r="M6" s="33"/>
-      <c r="N6" s="33"/>
-    </row>
-    <row r="7" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J6" s="36"/>
+      <c r="K6" s="36"/>
+      <c r="L6" s="38">
+        <v>25</v>
+      </c>
+      <c r="M6" s="38"/>
+      <c r="N6" s="38"/>
+      <c r="O6" s="33">
+        <v>14</v>
+      </c>
+      <c r="P6" s="33"/>
+      <c r="Q6" s="33"/>
+    </row>
+    <row r="7" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="32">
-        <v>42</v>
-      </c>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="30"/>
-    </row>
-    <row r="8" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="39">
+        <v>81</v>
+      </c>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="39"/>
+      <c r="L7" s="39"/>
+      <c r="M7" s="39"/>
+      <c r="N7" s="39"/>
+      <c r="O7" s="39"/>
+      <c r="P7" s="39"/>
+      <c r="Q7" s="39"/>
+    </row>
+    <row r="8" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1299,7 +1530,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1313,7 +1544,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -1327,7 +1558,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1344,7 +1575,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1361,7 +1592,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1375,7 +1606,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -1392,7 +1623,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1884,7 +2115,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>91</v>
       </c>
@@ -1895,7 +2126,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>93</v>
       </c>
@@ -1906,7 +2137,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>101</v>
       </c>
@@ -1916,8 +2147,11 @@
       <c r="L51" s="24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O51" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>102</v>
       </c>
@@ -1927,8 +2161,11 @@
       <c r="L52" s="24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O52" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>103</v>
       </c>
@@ -1938,8 +2175,11 @@
       <c r="L53" s="24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O53" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>104</v>
       </c>
@@ -1949,8 +2189,11 @@
       <c r="L54" s="24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O54" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>105</v>
       </c>
@@ -1960,8 +2203,11 @@
       <c r="L55" s="24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O55" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>106</v>
       </c>
@@ -1971,8 +2217,11 @@
       <c r="L56" s="24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O56" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>107</v>
       </c>
@@ -1982,8 +2231,11 @@
       <c r="L57" s="24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O57" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>108</v>
       </c>
@@ -1997,7 +2249,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>109</v>
       </c>
@@ -2008,7 +2260,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>110</v>
       </c>
@@ -2021,8 +2273,11 @@
       <c r="M60" s="25" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O60" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>111</v>
       </c>
@@ -2032,8 +2287,11 @@
       <c r="L61" s="24" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="O61" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>112</v>
       </c>
@@ -2047,7 +2305,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>113</v>
       </c>
@@ -2061,7 +2319,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>132</v>
       </c>
@@ -2072,7 +2330,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>134</v>
       </c>
@@ -2085,8 +2343,11 @@
       <c r="N65" s="26" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O65" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>136</v>
       </c>
@@ -2096,8 +2357,11 @@
       <c r="M66" s="25" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O66" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>138</v>
       </c>
@@ -2108,7 +2372,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>140</v>
       </c>
@@ -2122,7 +2386,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>142</v>
       </c>
@@ -2136,7 +2400,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>144</v>
       </c>
@@ -2146,8 +2410,11 @@
       <c r="M70" s="25" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O70" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>146</v>
       </c>
@@ -2161,7 +2428,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>148</v>
       </c>
@@ -2172,7 +2439,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>150</v>
       </c>
@@ -2183,19 +2450,225 @@
         <v>15</v>
       </c>
     </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>152</v>
+      </c>
+      <c r="B74" t="s">
+        <v>153</v>
+      </c>
+      <c r="N74" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>154</v>
+      </c>
+      <c r="B75" t="s">
+        <v>157</v>
+      </c>
+      <c r="N75" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>155</v>
+      </c>
+      <c r="B76" t="s">
+        <v>156</v>
+      </c>
+      <c r="N76" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>159</v>
+      </c>
+      <c r="B77" t="s">
+        <v>158</v>
+      </c>
+      <c r="N77" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>163</v>
+      </c>
+      <c r="B78" t="s">
+        <v>164</v>
+      </c>
+      <c r="O78" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>165</v>
+      </c>
+      <c r="B79" t="s">
+        <v>167</v>
+      </c>
+      <c r="O79" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>166</v>
+      </c>
+      <c r="B80" t="s">
+        <v>168</v>
+      </c>
+      <c r="O80" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>169</v>
+      </c>
+      <c r="B81" t="s">
+        <v>170</v>
+      </c>
+      <c r="O81" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>171</v>
+      </c>
+      <c r="B82" t="s">
+        <v>172</v>
+      </c>
+      <c r="O82" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>173</v>
+      </c>
+      <c r="B83" t="s">
+        <v>176</v>
+      </c>
+      <c r="O83" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="P83" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>174</v>
+      </c>
+      <c r="B84" t="s">
+        <v>175</v>
+      </c>
+      <c r="O84" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="P84" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>177</v>
+      </c>
+      <c r="B85" t="s">
+        <v>178</v>
+      </c>
+      <c r="P85" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>179</v>
+      </c>
+      <c r="B86" t="s">
+        <v>180</v>
+      </c>
+      <c r="P86" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>181</v>
+      </c>
+      <c r="B87" t="s">
+        <v>185</v>
+      </c>
+      <c r="P87" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>182</v>
+      </c>
+      <c r="B88" t="s">
+        <v>186</v>
+      </c>
+      <c r="P88" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>183</v>
+      </c>
+      <c r="B89" t="s">
+        <v>187</v>
+      </c>
+      <c r="P89" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>184</v>
+      </c>
+      <c r="B90" t="s">
+        <v>188</v>
+      </c>
+      <c r="P90" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>189</v>
+      </c>
+      <c r="B91" t="s">
+        <v>190</v>
+      </c>
+      <c r="P91" s="31" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
+    <mergeCell ref="C7:Q7"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="O6:Q6"/>
     <mergeCell ref="L1:N1"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="I6:K6"/>
     <mergeCell ref="F6:H6"/>
-    <mergeCell ref="C7:K7"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="I1:K1"/>
     <mergeCell ref="L6:N6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finished Verdant Forest Opponents. About to refactor all NPC data for easier management
</commit_message>
<xml_diff>
--- a/Opponent_Tracker.xlsx
+++ b/Opponent_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B45039-599A-485E-B279-47A4CCF1E17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84EA83B0-7A4D-400B-AE8C-49E9139A78F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28785" yWindow="0" windowWidth="28920" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="opponents_table" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="197">
   <si>
     <t>Opponent</t>
   </si>
@@ -593,6 +593,24 @@
   </si>
   <si>
     <t>Rocket Psychic Supremacy</t>
+  </si>
+  <si>
+    <t>Veteran Sylvester</t>
+  </si>
+  <si>
+    <t>Lost At Sea</t>
+  </si>
+  <si>
+    <t>Psychic Eli</t>
+  </si>
+  <si>
+    <t>Mind Control</t>
+  </si>
+  <si>
+    <t>Light Engineer Chase</t>
+  </si>
+  <si>
+    <t>Shock and Awe</t>
   </si>
 </sst>
 </file>
@@ -762,7 +780,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -855,6 +873,9 @@
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -874,7 +895,7 @@
     <xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -885,10 +906,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFC600EE"/>
       <color rgb="FFFFC901"/>
       <color rgb="FF3FBFFF"/>
       <color rgb="FFC3EA00"/>
-      <color rgb="FFC600EE"/>
       <color rgb="FFFFED01"/>
       <color rgb="FF55FE00"/>
       <color rgb="FF6600CC"/>
@@ -1225,7 +1246,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q91"/>
+  <dimension ref="A1:Q94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -1234,31 +1255,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C1" s="32" t="s">
+      <c r="C1" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32" t="s">
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32" t="s">
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32" t="s">
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32" t="s">
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="32"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="33"/>
     </row>
     <row r="2" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
@@ -1467,53 +1488,53 @@
       <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="34">
+      <c r="C6" s="35">
         <v>8</v>
       </c>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="37">
-        <v>15</v>
-      </c>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="35">
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="38">
+        <v>15</v>
+      </c>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="36">
         <v>19</v>
       </c>
-      <c r="J6" s="36"/>
-      <c r="K6" s="36"/>
-      <c r="L6" s="38">
+      <c r="J6" s="37"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="39">
         <v>25</v>
       </c>
-      <c r="M6" s="38"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="33">
+      <c r="M6" s="39"/>
+      <c r="N6" s="39"/>
+      <c r="O6" s="34">
         <v>14</v>
       </c>
-      <c r="P6" s="33"/>
-      <c r="Q6" s="33"/>
+      <c r="P6" s="34"/>
+      <c r="Q6" s="34"/>
     </row>
     <row r="7" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="32">
         <v>81</v>
       </c>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="39"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="39"/>
-      <c r="J7" s="39"/>
-      <c r="K7" s="39"/>
-      <c r="L7" s="39"/>
-      <c r="M7" s="39"/>
-      <c r="N7" s="39"/>
-      <c r="O7" s="39"/>
-      <c r="P7" s="39"/>
-      <c r="Q7" s="39"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="32"/>
+      <c r="N7" s="32"/>
+      <c r="O7" s="32"/>
+      <c r="P7" s="32"/>
+      <c r="Q7" s="32"/>
     </row>
     <row r="8" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2330,7 +2351,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>134</v>
       </c>
@@ -2347,7 +2368,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>136</v>
       </c>
@@ -2361,7 +2382,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>138</v>
       </c>
@@ -2372,7 +2393,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>140</v>
       </c>
@@ -2386,7 +2407,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>142</v>
       </c>
@@ -2400,7 +2421,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>144</v>
       </c>
@@ -2414,7 +2435,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>146</v>
       </c>
@@ -2428,7 +2449,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>148</v>
       </c>
@@ -2439,7 +2460,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>150</v>
       </c>
@@ -2450,7 +2471,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>152</v>
       </c>
@@ -2461,7 +2482,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>154</v>
       </c>
@@ -2472,7 +2493,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>155</v>
       </c>
@@ -2483,7 +2504,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>159</v>
       </c>
@@ -2494,7 +2515,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>163</v>
       </c>
@@ -2504,8 +2525,14 @@
       <c r="O78" s="30" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P78" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q78" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>165</v>
       </c>
@@ -2516,7 +2543,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>166</v>
       </c>
@@ -2527,7 +2554,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>169</v>
       </c>
@@ -2538,7 +2565,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>171</v>
       </c>
@@ -2549,7 +2576,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>173</v>
       </c>
@@ -2563,7 +2590,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>174</v>
       </c>
@@ -2577,7 +2604,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>177</v>
       </c>
@@ -2587,8 +2614,11 @@
       <c r="P85" s="31" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q85" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>179</v>
       </c>
@@ -2598,8 +2628,11 @@
       <c r="P86" s="31" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q86" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>181</v>
       </c>
@@ -2609,8 +2642,11 @@
       <c r="P87" s="31" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q87" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>182</v>
       </c>
@@ -2620,8 +2656,11 @@
       <c r="P88" s="31" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q88" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>183</v>
       </c>
@@ -2631,8 +2670,11 @@
       <c r="P89" s="31" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q89" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>184</v>
       </c>
@@ -2642,8 +2684,11 @@
       <c r="P90" s="31" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q90" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>189</v>
       </c>
@@ -2652,6 +2697,39 @@
       </c>
       <c r="P91" s="31" t="s">
         <v>15</v>
+      </c>
+      <c r="Q91" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>191</v>
+      </c>
+      <c r="B92" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q92" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>193</v>
+      </c>
+      <c r="B93" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q93" s="40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>195</v>
+      </c>
+      <c r="B94" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactored code to have prizes in a single constant file to make them easier to change.
</commit_message>
<xml_diff>
--- a/Opponent_Tracker.xlsx
+++ b/Opponent_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84EA83B0-7A4D-400B-AE8C-49E9139A78F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA36DD2C-463C-4BEB-83CE-82BC64AC99D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28785" yWindow="0" windowWidth="28920" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="opponents_table" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="197">
   <si>
     <t>Opponent</t>
   </si>
@@ -873,6 +873,9 @@
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -894,9 +897,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -906,15 +906,15 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF6600CC"/>
+      <color rgb="FFFF6600"/>
+      <color rgb="FF2D55FF"/>
       <color rgb="FFC600EE"/>
       <color rgb="FFFFC901"/>
       <color rgb="FF3FBFFF"/>
       <color rgb="FFC3EA00"/>
       <color rgb="FFFFED01"/>
       <color rgb="FF55FE00"/>
-      <color rgb="FF6600CC"/>
-      <color rgb="FFFF6600"/>
-      <color rgb="FF2D55FF"/>
       <color rgb="FF4F79FF"/>
     </mruColors>
   </colors>
@@ -1255,31 +1255,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C1" s="33" t="s">
+      <c r="C1" s="34" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33" t="s">
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33" t="s">
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34" t="s">
         <v>130</v>
       </c>
-      <c r="J1" s="33"/>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33" t="s">
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="M1" s="33"/>
-      <c r="N1" s="33"/>
-      <c r="O1" s="33" t="s">
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="P1" s="33"/>
-      <c r="Q1" s="33"/>
+      <c r="P1" s="34"/>
+      <c r="Q1" s="34"/>
     </row>
     <row r="2" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
@@ -1381,7 +1381,7 @@
         <v>7</v>
       </c>
       <c r="Q3" s="29">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1472,69 +1472,69 @@
         <v>11</v>
       </c>
       <c r="N5" s="23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O5" s="27">
         <v>19</v>
       </c>
       <c r="P5" s="28">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q5" s="29">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="35">
+      <c r="C6" s="36">
         <v>8</v>
       </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="38">
-        <v>15</v>
-      </c>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="36">
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="39">
+        <v>15</v>
+      </c>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="37">
         <v>19</v>
       </c>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
-      <c r="L6" s="39">
+      <c r="J6" s="38"/>
+      <c r="K6" s="38"/>
+      <c r="L6" s="40">
         <v>25</v>
       </c>
-      <c r="M6" s="39"/>
-      <c r="N6" s="39"/>
-      <c r="O6" s="34">
+      <c r="M6" s="40"/>
+      <c r="N6" s="40"/>
+      <c r="O6" s="35">
         <v>14</v>
       </c>
-      <c r="P6" s="34"/>
-      <c r="Q6" s="34"/>
+      <c r="P6" s="35"/>
+      <c r="Q6" s="35"/>
     </row>
     <row r="7" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="32">
+      <c r="C7" s="33">
         <v>81</v>
       </c>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="32"/>
-      <c r="K7" s="32"/>
-      <c r="L7" s="32"/>
-      <c r="M7" s="32"/>
-      <c r="N7" s="32"/>
-      <c r="O7" s="32"/>
-      <c r="P7" s="32"/>
-      <c r="Q7" s="32"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="33"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="33"/>
+      <c r="O7" s="33"/>
+      <c r="P7" s="33"/>
+      <c r="Q7" s="33"/>
     </row>
     <row r="8" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1595,6 +1595,9 @@
       <c r="I12" s="17" t="s">
         <v>15</v>
       </c>
+      <c r="L12" s="24" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -1612,6 +1615,9 @@
       <c r="I13" s="17" t="s">
         <v>15</v>
       </c>
+      <c r="L13" s="24" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -1643,6 +1649,9 @@
       <c r="J15" s="18" t="s">
         <v>15</v>
       </c>
+      <c r="M15" s="25" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="16" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1658,7 +1667,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1671,8 +1680,11 @@
       <c r="I17" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L17" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1685,8 +1697,11 @@
       <c r="I18" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L18" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -1705,8 +1720,14 @@
       <c r="J19" s="18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L19" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M19" s="25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1722,8 +1743,11 @@
       <c r="I20" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L20" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -1739,8 +1763,11 @@
       <c r="I21" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L21" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -1756,8 +1783,11 @@
       <c r="I22" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L22" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -1773,8 +1803,11 @@
       <c r="I23" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L23" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>100</v>
       </c>
@@ -1793,8 +1826,14 @@
       <c r="J24" s="18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L24" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M24" s="25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -1810,8 +1849,11 @@
       <c r="I25" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L25" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>47</v>
       </c>
@@ -1827,8 +1869,11 @@
       <c r="J26" s="18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M26" s="25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>49</v>
       </c>
@@ -1844,8 +1889,11 @@
       <c r="I27" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L27" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>51</v>
       </c>
@@ -1861,8 +1909,11 @@
       <c r="I28" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L28" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>53</v>
       </c>
@@ -1875,8 +1926,11 @@
       <c r="K29" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N29" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>55</v>
       </c>
@@ -1892,8 +1946,14 @@
       <c r="K30" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M30" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N30" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>57</v>
       </c>
@@ -1906,8 +1966,11 @@
       <c r="K31" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="N31" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>59</v>
       </c>
@@ -1917,8 +1980,11 @@
       <c r="I32" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L32" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>61</v>
       </c>
@@ -1928,8 +1994,11 @@
       <c r="I33" s="17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L33" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>63</v>
       </c>
@@ -1942,8 +2011,14 @@
       <c r="J34" s="18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L34" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M34" s="25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>65</v>
       </c>
@@ -1956,8 +2031,14 @@
       <c r="J35" s="18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L35" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M35" s="25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>67</v>
       </c>
@@ -1973,8 +2054,17 @@
       <c r="K36" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L36" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M36" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N36" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>69</v>
       </c>
@@ -1987,8 +2077,14 @@
       <c r="J37" s="18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L37" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M37" s="25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>71</v>
       </c>
@@ -2001,8 +2097,14 @@
       <c r="J38" s="18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L38" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M38" s="25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>73</v>
       </c>
@@ -2015,8 +2117,14 @@
       <c r="J39" s="18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L39" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M39" s="25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>96</v>
       </c>
@@ -2029,8 +2137,14 @@
       <c r="K40" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M40" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N40" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>76</v>
       </c>
@@ -2043,8 +2157,14 @@
       <c r="K41" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M41" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N41" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>78</v>
       </c>
@@ -2057,8 +2177,14 @@
       <c r="K42" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M42" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N42" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>80</v>
       </c>
@@ -2071,8 +2197,14 @@
       <c r="K43" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M43" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N43" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>82</v>
       </c>
@@ -2085,8 +2217,14 @@
       <c r="K44" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M44" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N44" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>95</v>
       </c>
@@ -2099,8 +2237,14 @@
       <c r="K45" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M45" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N45" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>85</v>
       </c>
@@ -2113,8 +2257,14 @@
       <c r="K46" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M46" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="N46" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>87</v>
       </c>
@@ -2124,8 +2274,11 @@
       <c r="K47" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="N47" s="26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>89</v>
       </c>
@@ -2133,6 +2286,9 @@
         <v>90</v>
       </c>
       <c r="K48" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="N48" s="26" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2146,6 +2302,9 @@
       <c r="K49" s="20" t="s">
         <v>15</v>
       </c>
+      <c r="N49" s="26" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
@@ -2157,6 +2316,9 @@
       <c r="K50" s="20" t="s">
         <v>15</v>
       </c>
+      <c r="N50" s="26" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
@@ -2528,7 +2690,7 @@
       <c r="P78" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="Q78" s="40" t="s">
+      <c r="Q78" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2614,7 +2776,7 @@
       <c r="P85" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="Q85" s="40" t="s">
+      <c r="Q85" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2628,7 +2790,7 @@
       <c r="P86" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="Q86" s="40" t="s">
+      <c r="Q86" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2642,7 +2804,7 @@
       <c r="P87" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="Q87" s="40" t="s">
+      <c r="Q87" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2656,7 +2818,7 @@
       <c r="P88" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="Q88" s="40" t="s">
+      <c r="Q88" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2670,7 +2832,7 @@
       <c r="P89" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="Q89" s="40" t="s">
+      <c r="Q89" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2684,7 +2846,7 @@
       <c r="P90" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="Q90" s="40" t="s">
+      <c r="Q90" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2698,7 +2860,7 @@
       <c r="P91" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="Q91" s="40" t="s">
+      <c r="Q91" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2709,7 +2871,7 @@
       <c r="B92" t="s">
         <v>192</v>
       </c>
-      <c r="Q92" s="40" t="s">
+      <c r="Q92" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2720,7 +2882,7 @@
       <c r="B93" t="s">
         <v>194</v>
       </c>
-      <c r="Q93" s="40" t="s">
+      <c r="Q93" s="32" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2730,6 +2892,9 @@
       </c>
       <c r="B94" t="s">
         <v>196</v>
+      </c>
+      <c r="Q94" s="32" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>